<commit_message>
Ajout des informations sur les nouveaux champs dans le fichier d'export
</commit_message>
<xml_diff>
--- a/public/templates/template_comparaison_EJ.xlsx
+++ b/public/templates/template_comparaison_EJ.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://catamaniacrm-my.sharepoint.com/personal/y_elhouakmi_catamania_com/Documents/Documents/DNum/Helios/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="47" documentId="8_{1007A4AD-03A1-49A6-9C75-414404E5FC40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2DB7AABD-2764-44C4-8FAA-27989E0C030D}"/>
+  <xr:revisionPtr revIDLastSave="66" documentId="8_{1007A4AD-03A1-49A6-9C75-414404E5FC40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9E8581BC-76FF-4787-9688-C26D4F9B9FE3}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="12" yWindow="12" windowWidth="23016" windowHeight="13656" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Lisez-moi" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="37">
   <si>
     <t>Indicateurs</t>
   </si>
@@ -1079,6 +1079,239 @@
       <t xml:space="preserve">
 Enquête « Bilan Social »- Agence technique de l’information sur l’hospitalisation (ATIH)
 Hélios collecte ces données depuis le SI mutualisé des ARS DIAMANT qui est un système décisionnel national permettant de stocker des informations provenant de plusieurs sources. DIAMANT : Décisionnel Inter-ARS pour la Maîtrise et l’Anticipation.</t>
+    </r>
+  </si>
+  <si>
+    <t>Fonds de roulement</t>
+  </si>
+  <si>
+    <t>Besoin en fonds de roulement</t>
+  </si>
+  <si>
+    <t>Tresorerie</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Le Besoin en Fonds de Roulement (BFR) traduit le besoin de financement du cycle d’exploitation.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Fréquence :</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Quotidienne
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Mode de calcul :</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Différence entre l’actif circulant et le passif circulant
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Source(s)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> : ANCRE (Application Nationale Compte financier Rapport infra-annuel Eprd) - Agence technique de l’information sur l’hospitalisation (ATIH)
+Hélios collecte ces données depuis le SI mutualisé des ARS DIAMANT « Décisionnel Inter-ARS pour la Maîtrise et l’Anticipation », outil décisionnel de pilotage centré sur la régulation de l’offre de soins, abordée sous les aspects des moyens humains, financiers, et productivité.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Le calcul du fonds de roulement permet d’apprécier l’adéquation des ressources aux emplois.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Fréquence :</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Quotidienne
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Mode de calcul :</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Différence entre les ressources stables (passif long terme) et les emplois stables (actif long terme)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Source(s) :</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+ANCRE (Application Nationale Compte financier Rapport infra-annuel Eprd) - Agence technique de l’information sur l’hospitalisation (ATIH)
+Hélios collecte ces données depuis le SI mutualisé des ARS DIAMANT « Décisionnel Inter-ARS pour la Maîtrise et l’Anticipation », outil décisionnel de pilotage centré sur la régulation de l’offre de soins, abordée sous les aspects des moyens humains, financiers, et productivité.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">La trésorerie désigne les liquidités ou quasi liquidités dont dispose l’établissement à un moment donné.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Fréquence :</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Quotidienne
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Mode de calcul :</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Trésorerie = Fonds de roulement - Besoin en fonds de roulement
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Source(s) :</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+ANCRE (Application Nationale Compte financier Rapport infra-annuel Eprd) - Agence technique de l’information sur l’hospitalisation (ATIH)
+Hélios collecte ces données depuis le SI mutualisé des ARS DIAMANT « Décisionnel Inter-ARS pour la Maîtrise et l’Anticipation », outil décisionnel de pilotage centré sur la régulation de l’offre de soins, abordée sous les aspects des moyens humains, financiers, et productivité.</t>
     </r>
   </si>
 </sst>
@@ -1148,13 +1381,13 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1495,15 +1728,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{587C9ED0-279B-44AC-9485-AC6832055B1B}">
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C20"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="20.875" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="187.625" style="2" customWidth="1"/>
+    <col min="1" max="1" width="20.8984375" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.09765625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="187.59765625" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1514,7 +1747,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="262.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="262.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
@@ -1525,94 +1758,94 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="157.5" x14ac:dyDescent="0.25">
-      <c r="A3" s="6" t="s">
+    <row r="3" spans="1:3" ht="156" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="157.5" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
+    <row r="4" spans="1:3" ht="156" x14ac:dyDescent="0.3">
+      <c r="A4" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="157.5" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
+    <row r="5" spans="1:3" ht="156" x14ac:dyDescent="0.3">
+      <c r="A5" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="173.25" x14ac:dyDescent="0.25">
-      <c r="A6" s="6" t="s">
+    <row r="6" spans="1:3" ht="171.6" x14ac:dyDescent="0.3">
+      <c r="A6" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="173.25" x14ac:dyDescent="0.25">
-      <c r="A7" s="6" t="s">
+    <row r="7" spans="1:3" ht="171.6" x14ac:dyDescent="0.3">
+      <c r="A7" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="5" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="5"/>
-      <c r="C9" s="4"/>
+      <c r="B9" s="6"/>
+      <c r="C9" s="5"/>
     </row>
-    <row r="10" spans="1:3" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="5"/>
-      <c r="C10" s="4"/>
+      <c r="B10" s="6"/>
+      <c r="C10" s="5"/>
     </row>
-    <row r="11" spans="1:3" ht="188.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" ht="188.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="5"/>
-      <c r="C11" s="4"/>
+      <c r="B11" s="6"/>
+      <c r="C11" s="5"/>
     </row>
-    <row r="12" spans="1:3" ht="180" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="180" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -1623,39 +1856,39 @@
         <v>13</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="4" t="s">
+    <row r="13" spans="1:3" ht="409.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="5" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="144" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="4"/>
-      <c r="B14" s="5"/>
-      <c r="C14" s="4"/>
+    <row r="14" spans="1:3" ht="144" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="5"/>
+      <c r="B14" s="6"/>
+      <c r="C14" s="5"/>
     </row>
-    <row r="15" spans="1:3" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="4" t="s">
+    <row r="15" spans="1:3" ht="409.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="5" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="100.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="4"/>
-      <c r="B16" s="5"/>
-      <c r="C16" s="4"/>
+    <row r="16" spans="1:3" ht="100.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="5"/>
+      <c r="B16" s="6"/>
+      <c r="C16" s="5"/>
     </row>
-    <row r="17" spans="1:3" ht="257.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" ht="286.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>18</v>
       </c>
@@ -1664,6 +1897,39 @@
       </c>
       <c r="C17" s="3" t="s">
         <v>20</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="249.6" x14ac:dyDescent="0.3">
+      <c r="A18" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="218.4" x14ac:dyDescent="0.3">
+      <c r="A19" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="249.6" x14ac:dyDescent="0.3">
+      <c r="A20" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -1685,7 +1951,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Ajout des informations sur les nouveaux champs dans le fichier d'export (#1079)
* Ajout des informations sur les nouveaux champs dans le fichier d'export

* Update du changelog
</commit_message>
<xml_diff>
--- a/public/templates/template_comparaison_EJ.xlsx
+++ b/public/templates/template_comparaison_EJ.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://catamaniacrm-my.sharepoint.com/personal/y_elhouakmi_catamania_com/Documents/Documents/DNum/Helios/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="47" documentId="8_{1007A4AD-03A1-49A6-9C75-414404E5FC40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2DB7AABD-2764-44C4-8FAA-27989E0C030D}"/>
+  <xr:revisionPtr revIDLastSave="66" documentId="8_{1007A4AD-03A1-49A6-9C75-414404E5FC40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9E8581BC-76FF-4787-9688-C26D4F9B9FE3}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="12" yWindow="12" windowWidth="23016" windowHeight="13656" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Lisez-moi" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="37">
   <si>
     <t>Indicateurs</t>
   </si>
@@ -1079,6 +1079,239 @@
       <t xml:space="preserve">
 Enquête « Bilan Social »- Agence technique de l’information sur l’hospitalisation (ATIH)
 Hélios collecte ces données depuis le SI mutualisé des ARS DIAMANT qui est un système décisionnel national permettant de stocker des informations provenant de plusieurs sources. DIAMANT : Décisionnel Inter-ARS pour la Maîtrise et l’Anticipation.</t>
+    </r>
+  </si>
+  <si>
+    <t>Fonds de roulement</t>
+  </si>
+  <si>
+    <t>Besoin en fonds de roulement</t>
+  </si>
+  <si>
+    <t>Tresorerie</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Le Besoin en Fonds de Roulement (BFR) traduit le besoin de financement du cycle d’exploitation.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Fréquence :</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Quotidienne
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Mode de calcul :</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Différence entre l’actif circulant et le passif circulant
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Source(s)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> : ANCRE (Application Nationale Compte financier Rapport infra-annuel Eprd) - Agence technique de l’information sur l’hospitalisation (ATIH)
+Hélios collecte ces données depuis le SI mutualisé des ARS DIAMANT « Décisionnel Inter-ARS pour la Maîtrise et l’Anticipation », outil décisionnel de pilotage centré sur la régulation de l’offre de soins, abordée sous les aspects des moyens humains, financiers, et productivité.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Le calcul du fonds de roulement permet d’apprécier l’adéquation des ressources aux emplois.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Fréquence :</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Quotidienne
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Mode de calcul :</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Différence entre les ressources stables (passif long terme) et les emplois stables (actif long terme)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Source(s) :</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+ANCRE (Application Nationale Compte financier Rapport infra-annuel Eprd) - Agence technique de l’information sur l’hospitalisation (ATIH)
+Hélios collecte ces données depuis le SI mutualisé des ARS DIAMANT « Décisionnel Inter-ARS pour la Maîtrise et l’Anticipation », outil décisionnel de pilotage centré sur la régulation de l’offre de soins, abordée sous les aspects des moyens humains, financiers, et productivité.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">La trésorerie désigne les liquidités ou quasi liquidités dont dispose l’établissement à un moment donné.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Fréquence :</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Quotidienne
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Mode de calcul :</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Trésorerie = Fonds de roulement - Besoin en fonds de roulement
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Source(s) :</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+ANCRE (Application Nationale Compte financier Rapport infra-annuel Eprd) - Agence technique de l’information sur l’hospitalisation (ATIH)
+Hélios collecte ces données depuis le SI mutualisé des ARS DIAMANT « Décisionnel Inter-ARS pour la Maîtrise et l’Anticipation », outil décisionnel de pilotage centré sur la régulation de l’offre de soins, abordée sous les aspects des moyens humains, financiers, et productivité.</t>
     </r>
   </si>
 </sst>
@@ -1148,13 +1381,13 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1495,15 +1728,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{587C9ED0-279B-44AC-9485-AC6832055B1B}">
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C20"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="20.875" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="187.625" style="2" customWidth="1"/>
+    <col min="1" max="1" width="20.8984375" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.09765625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="187.59765625" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1514,7 +1747,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="262.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="262.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
@@ -1525,94 +1758,94 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="157.5" x14ac:dyDescent="0.25">
-      <c r="A3" s="6" t="s">
+    <row r="3" spans="1:3" ht="156" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="157.5" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
+    <row r="4" spans="1:3" ht="156" x14ac:dyDescent="0.3">
+      <c r="A4" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="157.5" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
+    <row r="5" spans="1:3" ht="156" x14ac:dyDescent="0.3">
+      <c r="A5" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="173.25" x14ac:dyDescent="0.25">
-      <c r="A6" s="6" t="s">
+    <row r="6" spans="1:3" ht="171.6" x14ac:dyDescent="0.3">
+      <c r="A6" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="173.25" x14ac:dyDescent="0.25">
-      <c r="A7" s="6" t="s">
+    <row r="7" spans="1:3" ht="171.6" x14ac:dyDescent="0.3">
+      <c r="A7" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="4" t="s">
         <v>7</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="47.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="5" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="5"/>
-      <c r="C9" s="4"/>
+      <c r="B9" s="6"/>
+      <c r="C9" s="5"/>
     </row>
-    <row r="10" spans="1:3" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" ht="46.8" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="5"/>
-      <c r="C10" s="4"/>
+      <c r="B10" s="6"/>
+      <c r="C10" s="5"/>
     </row>
-    <row r="11" spans="1:3" ht="188.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" ht="188.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="5"/>
-      <c r="C11" s="4"/>
+      <c r="B11" s="6"/>
+      <c r="C11" s="5"/>
     </row>
-    <row r="12" spans="1:3" ht="180" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="180" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -1623,39 +1856,39 @@
         <v>13</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="4" t="s">
+    <row r="13" spans="1:3" ht="409.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="5" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="144" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="4"/>
-      <c r="B14" s="5"/>
-      <c r="C14" s="4"/>
+    <row r="14" spans="1:3" ht="144" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="5"/>
+      <c r="B14" s="6"/>
+      <c r="C14" s="5"/>
     </row>
-    <row r="15" spans="1:3" ht="409.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="4" t="s">
+    <row r="15" spans="1:3" ht="409.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="5" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="100.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="4"/>
-      <c r="B16" s="5"/>
-      <c r="C16" s="4"/>
+    <row r="16" spans="1:3" ht="100.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="5"/>
+      <c r="B16" s="6"/>
+      <c r="C16" s="5"/>
     </row>
-    <row r="17" spans="1:3" ht="257.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" ht="286.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>18</v>
       </c>
@@ -1664,6 +1897,39 @@
       </c>
       <c r="C17" s="3" t="s">
         <v>20</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="249.6" x14ac:dyDescent="0.3">
+      <c r="A18" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="218.4" x14ac:dyDescent="0.3">
+      <c r="A19" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="249.6" x14ac:dyDescent="0.3">
+      <c r="A20" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -1685,7 +1951,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>